<commit_message>
feat: Add GreenSIG data processing and reporting scripts
- Introduced `rapport_greensig_dsl.py` to process real data from `db_greensig` through the GreenSIG adapter, generating a detailed report in CSV and Markdown formats.
- Created `rapport_dsl.md` and `rapport_dsl.csv` to document task-level results and summaries.
- Implemented shared utilities in `base.py` for loading mission contracts and extracting code blocks from LLM responses.
- Enhanced error handling and reporting for task translation failures, including detailed validation error messages.
</commit_message>
<xml_diff>
--- a/docs/dsl/gabarit_ingestion_trco.xlsx
+++ b/docs/dsl/gabarit_ingestion_trco.xlsx
@@ -122,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -148,6 +148,9 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -9617,11 +9620,27 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="8" t="n"/>
-      <c r="B6" s="8" t="n"/>
-      <c r="C6" s="8" t="n"/>
-      <c r="D6" s="8" t="n"/>
+    <row r="6" ht="60" customHeight="1">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>Déterminer, à partir des compétences des opérateurs, quelles équipes sont compatibles avec les tâches jamais affectées (228/1007 sur le dernier export, 23 %) — pas les affecter nous-mêmes, juste leur donner des candidates pour que le solveur choisisse.</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Contrainte supplémentaire</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>api_users_competence/api_users_competenceoperateur existe côté GreenSIG mais n'est relié aux types de tâche par aucune clé fiable (noms proches mais pas identiques, ex. "Tonte" vs "Utilisation de tondeuse") — demande un mappage type_tache↔compétence validé à la main avant d'être exploitable.</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Constat interne — adapters/greensig/rapport_dsl.md, 2026-07-16</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="n"/>

</xml_diff>